<commit_message>
fixed a bug in fixed intertie capacity factors
</commit_message>
<xml_diff>
--- a/input_files/capacity_limits.xlsx
+++ b/input_files/capacity_limits.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://utoronto-my.sharepoint.com/personal/ian_elder_mail_utoronto_ca/Documents/Documents/TEMOA/CODERS scripts/input_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="128" documentId="8_{AD9299FD-BE0E-4A8B-BE4E-54B5B8BEA38F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA1DC616-41B6-4427-8CE5-7E878A34A2B5}"/>
+  <xr:revisionPtr revIDLastSave="139" documentId="8_{AD9299FD-BE0E-4A8B-BE4E-54B5B8BEA38F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08131A89-F3AB-48F6-BB95-5DB5CDCD5232}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{34B1FE10-2B49-41F7-8CAC-48335CB056E6}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="47">
   <si>
     <t>tech</t>
   </si>
@@ -135,9 +135,6 @@
     <t>New biogas generation potential for ontario</t>
   </si>
   <si>
-    <t>New hydroelectric generation potential for ontario. Half assumed to be run-of-river, the other half daily storage.</t>
-  </si>
-  <si>
     <t>Assumed that Ontario does not have requisite geology for geothermal generation</t>
   </si>
   <si>
@@ -166,6 +163,18 @@
   </si>
   <si>
     <t>E_HYD_ROR-NEW-5</t>
+  </si>
+  <si>
+    <t>New hydroelectric generation potential for ontario. Half assumed to be run-of-river, the other half daily storage (similar to existing).</t>
+  </si>
+  <si>
+    <t>E_COAL-NEW</t>
+  </si>
+  <si>
+    <t>E_COAL_CCS-NEW</t>
+  </si>
+  <si>
+    <t>Assume no new coal generation</t>
   </si>
 </sst>
 </file>
@@ -524,7 +533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9D36A0F-FD90-42AA-87C7-33795DBA1E16}">
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.140625" customWidth="1"/>
@@ -1168,7 +1177,7 @@
         <v>2500</v>
       </c>
       <c r="H25" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="I25">
         <v>2</v>
@@ -1179,7 +1188,7 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -1200,12 +1209,12 @@
         <v>0</v>
       </c>
       <c r="H26" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -1226,7 +1235,7 @@
         <v>0</v>
       </c>
       <c r="H27" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I27">
         <v>1</v>
@@ -1237,7 +1246,7 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B28">
         <v>0</v>
@@ -1258,7 +1267,7 @@
         <v>0</v>
       </c>
       <c r="H28" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I28">
         <v>1</v>
@@ -1269,7 +1278,7 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B29">
         <v>500</v>
@@ -1290,7 +1299,7 @@
         <v>500</v>
       </c>
       <c r="H29" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="I29">
         <v>2</v>
@@ -1301,7 +1310,7 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B30">
         <v>500</v>
@@ -1322,7 +1331,7 @@
         <v>500</v>
       </c>
       <c r="H30" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="I30">
         <v>2</v>
@@ -1333,7 +1342,7 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B31">
         <v>500</v>
@@ -1354,7 +1363,7 @@
         <v>500</v>
       </c>
       <c r="H31" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="I31">
         <v>2</v>
@@ -1365,7 +1374,7 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B32">
         <v>500</v>
@@ -1386,7 +1395,7 @@
         <v>500</v>
       </c>
       <c r="H32" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="I32">
         <v>2</v>
@@ -1397,34 +1406,86 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>42</v>
+      </c>
+      <c r="B33">
+        <v>500</v>
+      </c>
+      <c r="C33">
+        <v>500</v>
+      </c>
+      <c r="D33">
+        <v>500</v>
+      </c>
+      <c r="E33">
+        <v>500</v>
+      </c>
+      <c r="F33">
+        <v>500</v>
+      </c>
+      <c r="G33">
+        <v>500</v>
+      </c>
+      <c r="H33" t="s">
         <v>43</v>
-      </c>
-      <c r="B33">
-        <v>500</v>
-      </c>
-      <c r="C33">
-        <v>500</v>
-      </c>
-      <c r="D33">
-        <v>500</v>
-      </c>
-      <c r="E33">
-        <v>500</v>
-      </c>
-      <c r="F33">
-        <v>500</v>
-      </c>
-      <c r="G33">
-        <v>500</v>
-      </c>
-      <c r="H33" t="s">
-        <v>33</v>
       </c>
       <c r="I33">
         <v>2</v>
       </c>
       <c r="J33" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>44</v>
+      </c>
+      <c r="B34">
+        <v>0</v>
+      </c>
+      <c r="C34">
+        <v>0</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+      <c r="E34">
+        <v>0</v>
+      </c>
+      <c r="F34">
+        <v>0</v>
+      </c>
+      <c r="G34">
+        <v>0</v>
+      </c>
+      <c r="H34" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>45</v>
+      </c>
+      <c r="B35">
+        <v>0</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
+      </c>
+      <c r="G35">
+        <v>0</v>
+      </c>
+      <c r="H35" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>